<commit_message>
Update ProductData.xlsx with new test data
</commit_message>
<xml_diff>
--- a/test_data/ProductData.xlsx
+++ b/test_data/ProductData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <r>
       <rPr>
@@ -103,9 +103,6 @@
   </si>
   <si>
     <t>Serving</t>
-  </si>
-  <si>
-    <t>water</t>
   </si>
 </sst>
 </file>
@@ -562,7 +559,7 @@
         <v>181</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" t="b">
         <v>0</v>

</xml_diff>